<commit_message>
Update test cases with Playwright results
</commit_message>
<xml_diff>
--- a/projects/NEXT_forum/Test-Case/NEXT-forum_Test-Case.xlsx
+++ b/projects/NEXT_forum/Test-Case/NEXT-forum_Test-Case.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\소연\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="4575" windowWidth="28800" windowHeight="11025"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38370" windowHeight="9000" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenario" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="285">
   <si>
     <t>ID</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1137,6 +1137,14 @@
   </si>
   <si>
     <t>GitHub 계정 정보 입력</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>로그아웃 자동화 테스트 미검증(수동 테스트로 확인)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Playwright 테스트에서도 중복 아이디로 회원가입이 완료되는 것을 확인함.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1364,21 +1372,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1391,13 +1396,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1752,18 +1760,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="26.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>254</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -1783,7 +1791,7 @@
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="22" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -1797,7 +1805,7 @@
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="14"/>
+      <c r="B4" s="22"/>
       <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1809,7 +1817,7 @@
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="14"/>
+      <c r="B5" s="22"/>
       <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
@@ -1821,7 +1829,7 @@
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="22" t="s">
         <v>35</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -1835,7 +1843,7 @@
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="14"/>
+      <c r="B7" s="22"/>
       <c r="C7" s="1" t="s">
         <v>37</v>
       </c>
@@ -1847,7 +1855,7 @@
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="14"/>
+      <c r="B8" s="22"/>
       <c r="C8" s="1" t="s">
         <v>39</v>
       </c>
@@ -1859,7 +1867,7 @@
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="14"/>
+      <c r="B9" s="22"/>
       <c r="C9" s="1" t="s">
         <v>12</v>
       </c>
@@ -1871,7 +1879,7 @@
       <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="14"/>
+      <c r="B10" s="22"/>
       <c r="C10" s="1" t="s">
         <v>41</v>
       </c>
@@ -1883,7 +1891,7 @@
       <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="14"/>
+      <c r="B11" s="22"/>
       <c r="C11" s="1" t="s">
         <v>44</v>
       </c>
@@ -1895,7 +1903,7 @@
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="14"/>
+      <c r="B12" s="22"/>
       <c r="C12" s="1" t="s">
         <v>46</v>
       </c>
@@ -1907,7 +1915,7 @@
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="22" t="s">
         <v>42</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -1921,7 +1929,7 @@
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="14"/>
+      <c r="B14" s="22"/>
       <c r="C14" s="1" t="s">
         <v>43</v>
       </c>
@@ -1933,7 +1941,7 @@
       <c r="A15" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="22" t="s">
         <v>47</v>
       </c>
       <c r="C15" s="1" t="s">
@@ -1947,7 +1955,7 @@
       <c r="A16" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="14"/>
+      <c r="B16" s="22"/>
       <c r="C16" s="1" t="s">
         <v>50</v>
       </c>
@@ -1959,7 +1967,7 @@
       <c r="A17" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="14"/>
+      <c r="B17" s="22"/>
       <c r="C17" s="1" t="s">
         <v>52</v>
       </c>
@@ -1971,7 +1979,7 @@
       <c r="A18" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="14"/>
+      <c r="B18" s="22"/>
       <c r="C18" s="1" t="s">
         <v>54</v>
       </c>
@@ -1983,7 +1991,7 @@
       <c r="A19" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="14"/>
+      <c r="B19" s="22"/>
       <c r="C19" s="1" t="s">
         <v>56</v>
       </c>
@@ -1995,7 +2003,7 @@
       <c r="A20" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="14"/>
+      <c r="B20" s="22"/>
       <c r="C20" s="1" t="s">
         <v>57</v>
       </c>
@@ -2007,7 +2015,7 @@
       <c r="A21" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="14"/>
+      <c r="B21" s="22"/>
       <c r="C21" s="1" t="s">
         <v>59</v>
       </c>
@@ -2019,7 +2027,7 @@
       <c r="A22" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="14"/>
+      <c r="B22" s="22"/>
       <c r="C22" s="1" t="s">
         <v>62</v>
       </c>
@@ -2031,7 +2039,7 @@
       <c r="A23" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="14"/>
+      <c r="B23" s="22"/>
       <c r="C23" s="1" t="s">
         <v>63</v>
       </c>
@@ -2043,7 +2051,7 @@
       <c r="A24" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="14"/>
+      <c r="B24" s="22"/>
       <c r="C24" s="1" t="s">
         <v>65</v>
       </c>
@@ -2055,7 +2063,7 @@
       <c r="A25" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="14"/>
+      <c r="B25" s="22"/>
       <c r="C25" s="1" t="s">
         <v>67</v>
       </c>
@@ -2067,7 +2075,7 @@
       <c r="A26" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="14"/>
+      <c r="B26" s="22"/>
       <c r="C26" s="1" t="s">
         <v>69</v>
       </c>
@@ -2079,7 +2087,7 @@
       <c r="A27" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="14"/>
+      <c r="B27" s="22"/>
       <c r="C27" s="1" t="s">
         <v>71</v>
       </c>
@@ -2091,7 +2099,7 @@
       <c r="A28" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B28" s="14"/>
+      <c r="B28" s="22"/>
       <c r="C28" s="1" t="s">
         <v>83</v>
       </c>
@@ -2103,7 +2111,7 @@
       <c r="A29" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B29" s="14"/>
+      <c r="B29" s="22"/>
       <c r="C29" s="1" t="s">
         <v>78</v>
       </c>
@@ -2115,7 +2123,7 @@
       <c r="A30" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B30" s="14"/>
+      <c r="B30" s="22"/>
       <c r="C30" s="1" t="s">
         <v>75</v>
       </c>
@@ -2127,7 +2135,7 @@
       <c r="A31" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B31" s="14"/>
+      <c r="B31" s="22"/>
       <c r="C31" s="1" t="s">
         <v>82</v>
       </c>
@@ -2139,7 +2147,7 @@
       <c r="A32" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B32" s="14"/>
+      <c r="B32" s="22"/>
       <c r="C32" s="1" t="s">
         <v>79</v>
       </c>
@@ -2151,7 +2159,7 @@
       <c r="A33" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B33" s="14"/>
+      <c r="B33" s="22"/>
       <c r="C33" s="1" t="s">
         <v>81</v>
       </c>
@@ -2163,7 +2171,7 @@
       <c r="A34" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B34" s="14"/>
+      <c r="B34" s="22"/>
       <c r="C34" s="1" t="s">
         <v>85</v>
       </c>
@@ -2175,7 +2183,7 @@
       <c r="A35" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B35" s="14"/>
+      <c r="B35" s="22"/>
       <c r="C35" s="1" t="s">
         <v>87</v>
       </c>
@@ -2187,7 +2195,7 @@
       <c r="A36" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B36" s="14" t="s">
+      <c r="B36" s="22" t="s">
         <v>89</v>
       </c>
       <c r="C36" s="1" t="s">
@@ -2201,7 +2209,7 @@
       <c r="A37" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B37" s="14"/>
+      <c r="B37" s="22"/>
       <c r="C37" s="1" t="s">
         <v>92</v>
       </c>
@@ -2213,7 +2221,7 @@
       <c r="A38" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B38" s="14"/>
+      <c r="B38" s="22"/>
       <c r="C38" s="1" t="s">
         <v>94</v>
       </c>
@@ -2225,7 +2233,7 @@
       <c r="A39" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B39" s="14"/>
+      <c r="B39" s="22"/>
       <c r="C39" s="1" t="s">
         <v>96</v>
       </c>
@@ -2261,22 +2269,23 @@
     <col min="6" max="6" width="35" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31.375" customWidth="1"/>
     <col min="8" max="9" width="72.625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="49.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="26.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>255</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="22"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="21"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -2320,25 +2329,25 @@
       <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="E3" s="23" t="s">
+      <c r="E3" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="14" t="s">
         <v>257</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="14" t="s">
         <v>273</v>
       </c>
-      <c r="H3" s="23" t="s">
+      <c r="H3" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="I3" s="23" t="s">
+      <c r="I3" s="16" t="s">
         <v>124</v>
       </c>
       <c r="J3" s="1" t="s">
@@ -2353,24 +2362,24 @@
       <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="14"/>
-      <c r="D4" s="23" t="s">
+      <c r="C4" s="22"/>
+      <c r="D4" s="16" t="s">
         <v>166</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="14" t="s">
         <v>273</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="I4" s="23" t="s">
-        <v>124</v>
+      <c r="I4" s="16" t="s">
+        <v>284</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>165</v>
@@ -2389,23 +2398,23 @@
       <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="23" t="s">
+      <c r="C5" s="22"/>
+      <c r="D5" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="G5" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="I5" s="23" t="s">
+      <c r="I5" s="16" t="s">
         <v>171</v>
       </c>
       <c r="J5" s="1" t="s">
@@ -2420,25 +2429,25 @@
       <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="23" t="s">
+      <c r="D6" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="E6" s="23" t="s">
+      <c r="E6" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="14" t="s">
         <v>260</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="14" t="s">
         <v>274</v>
       </c>
-      <c r="H6" s="23" t="s">
+      <c r="H6" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="I6" s="23" t="s">
+      <c r="I6" s="16" t="s">
         <v>204</v>
       </c>
       <c r="J6" s="1" t="s">
@@ -2455,23 +2464,23 @@
       <c r="B7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="14"/>
-      <c r="D7" s="23" t="s">
+      <c r="C7" s="22"/>
+      <c r="D7" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="14" t="s">
         <v>261</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" s="14" t="s">
         <v>275</v>
       </c>
-      <c r="H7" s="23" t="s">
+      <c r="H7" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="I7" s="23" t="s">
+      <c r="I7" s="16" t="s">
         <v>206</v>
       </c>
       <c r="J7" s="1" t="s">
@@ -2486,23 +2495,23 @@
       <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="23" t="s">
+      <c r="C8" s="22"/>
+      <c r="D8" s="16" t="s">
         <v>184</v>
       </c>
-      <c r="E8" s="23" t="s">
+      <c r="E8" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="14" t="s">
         <v>262</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="14" t="s">
         <v>276</v>
       </c>
-      <c r="H8" s="23" t="s">
+      <c r="H8" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="I8" s="23" t="s">
+      <c r="I8" s="16" t="s">
         <v>206</v>
       </c>
       <c r="J8" s="1" t="s">
@@ -2517,23 +2526,23 @@
       <c r="B9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="23" t="s">
+      <c r="C9" s="22"/>
+      <c r="D9" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="14" t="s">
         <v>263</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="G9" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="H9" s="23" t="s">
+      <c r="H9" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="I9" s="23" t="s">
+      <c r="I9" s="16" t="s">
         <v>206</v>
       </c>
       <c r="J9" s="1" t="s">
@@ -2548,23 +2557,23 @@
       <c r="B10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="23" t="s">
+      <c r="C10" s="22"/>
+      <c r="D10" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="E10" s="23" t="s">
+      <c r="E10" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="14" t="s">
         <v>277</v>
       </c>
-      <c r="H10" s="23" t="s">
+      <c r="H10" s="16" t="s">
         <v>187</v>
       </c>
-      <c r="I10" s="23" t="s">
+      <c r="I10" s="16" t="s">
         <v>187</v>
       </c>
       <c r="J10" s="1" t="s">
@@ -2579,23 +2588,23 @@
       <c r="B11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="23" t="s">
+      <c r="C11" s="22"/>
+      <c r="D11" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="E11" s="23" t="s">
+      <c r="E11" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="14" t="s">
         <v>188</v>
       </c>
       <c r="G11" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H11" s="23" t="s">
+      <c r="H11" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="I11" s="23" t="s">
+      <c r="I11" s="16" t="s">
         <v>209</v>
       </c>
       <c r="J11" s="1" t="s">
@@ -2610,23 +2619,23 @@
       <c r="B12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="23" t="s">
+      <c r="C12" s="22"/>
+      <c r="D12" s="16" t="s">
         <v>193</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="E12" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="G12" s="23" t="s">
+      <c r="G12" s="16" t="s">
         <v>282</v>
       </c>
-      <c r="H12" s="25" t="s">
+      <c r="H12" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="I12" s="25" t="s">
+      <c r="I12" s="18" t="s">
         <v>204</v>
       </c>
       <c r="J12" s="1" t="s">
@@ -2643,25 +2652,25 @@
       <c r="B13" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="16" t="s">
         <v>198</v>
       </c>
-      <c r="E13" s="23" t="s">
+      <c r="E13" s="16" t="s">
         <v>195</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="16" t="s">
         <v>196</v>
       </c>
       <c r="G13" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H13" s="23" t="s">
+      <c r="H13" s="16" t="s">
         <v>199</v>
       </c>
-      <c r="I13" s="23" t="s">
+      <c r="I13" s="16" t="s">
         <v>205</v>
       </c>
       <c r="J13" s="1" t="s">
@@ -2678,23 +2687,23 @@
       <c r="B14" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="23" t="s">
+      <c r="C14" s="22"/>
+      <c r="D14" s="16" t="s">
         <v>203</v>
       </c>
-      <c r="E14" s="23" t="s">
+      <c r="E14" s="16" t="s">
         <v>207</v>
       </c>
-      <c r="F14" s="23" t="s">
+      <c r="F14" s="16" t="s">
         <v>196</v>
       </c>
       <c r="G14" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H14" s="23" t="s">
+      <c r="H14" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="I14" s="23" t="s">
+      <c r="I14" s="16" t="s">
         <v>201</v>
       </c>
       <c r="J14" s="1" t="s">
@@ -2709,25 +2718,25 @@
       <c r="B15" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="E15" s="23" t="s">
+      <c r="E15" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="F15" s="23" t="s">
+      <c r="F15" s="16" t="s">
         <v>210</v>
       </c>
       <c r="G15" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H15" s="23" t="s">
+      <c r="H15" s="16" t="s">
         <v>214</v>
       </c>
-      <c r="I15" s="23" t="s">
+      <c r="I15" s="16" t="s">
         <v>212</v>
       </c>
       <c r="J15" s="1" t="s">
@@ -2742,23 +2751,23 @@
       <c r="B16" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="23" t="s">
+      <c r="C16" s="22"/>
+      <c r="D16" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="E16" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="F16" s="23" t="s">
+      <c r="F16" s="16" t="s">
         <v>215</v>
       </c>
       <c r="G16" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H16" s="23" t="s">
+      <c r="H16" s="16" t="s">
         <v>213</v>
       </c>
-      <c r="I16" s="23" t="s">
+      <c r="I16" s="16" t="s">
         <v>213</v>
       </c>
       <c r="J16" s="1" t="s">
@@ -2773,11 +2782,11 @@
       <c r="B17" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="23" t="s">
+      <c r="C17" s="22"/>
+      <c r="D17" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="16" t="s">
         <v>216</v>
       </c>
       <c r="F17" s="12" t="s">
@@ -2786,10 +2795,10 @@
       <c r="G17" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H17" s="23" t="s">
+      <c r="H17" s="16" t="s">
         <v>222</v>
       </c>
-      <c r="I17" s="23" t="s">
+      <c r="I17" s="16" t="s">
         <v>217</v>
       </c>
       <c r="J17" s="1" t="s">
@@ -2804,23 +2813,23 @@
       <c r="B18" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="23" t="s">
+      <c r="C18" s="22"/>
+      <c r="D18" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="E18" s="23" t="s">
+      <c r="E18" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="F18" s="23" t="s">
+      <c r="F18" s="16" t="s">
         <v>215</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H18" s="23" t="s">
+      <c r="H18" s="16" t="s">
         <v>229</v>
       </c>
-      <c r="I18" s="23" t="s">
+      <c r="I18" s="16" t="s">
         <v>229</v>
       </c>
       <c r="J18" s="11" t="s">
@@ -2835,23 +2844,23 @@
       <c r="B19" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="23" t="s">
+      <c r="C19" s="22"/>
+      <c r="D19" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="23" t="s">
+      <c r="E19" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="F19" s="23" t="s">
+      <c r="F19" s="16" t="s">
         <v>218</v>
       </c>
       <c r="G19" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H19" s="23" t="s">
+      <c r="H19" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="I19" s="23" t="s">
+      <c r="I19" s="16" t="s">
         <v>201</v>
       </c>
       <c r="J19" s="1" t="s">
@@ -2866,23 +2875,23 @@
       <c r="B20" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="23" t="s">
+      <c r="C20" s="22"/>
+      <c r="D20" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="E20" s="23" t="s">
+      <c r="E20" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="F20" s="23" t="s">
+      <c r="F20" s="16" t="s">
         <v>218</v>
       </c>
       <c r="G20" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H20" s="23" t="s">
+      <c r="H20" s="16" t="s">
         <v>219</v>
       </c>
-      <c r="I20" s="23" t="s">
+      <c r="I20" s="16" t="s">
         <v>219</v>
       </c>
       <c r="J20" s="1" t="s">
@@ -2897,23 +2906,23 @@
       <c r="B21" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="14"/>
-      <c r="D21" s="23" t="s">
+      <c r="C21" s="22"/>
+      <c r="D21" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="E21" s="23" t="s">
+      <c r="E21" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="F21" s="18" t="s">
+      <c r="F21" s="14" t="s">
         <v>266</v>
       </c>
-      <c r="G21" s="18" t="s">
+      <c r="G21" s="14" t="s">
         <v>278</v>
       </c>
-      <c r="H21" s="23" t="s">
+      <c r="H21" s="16" t="s">
         <v>221</v>
       </c>
-      <c r="I21" s="23" t="s">
+      <c r="I21" s="16" t="s">
         <v>221</v>
       </c>
       <c r="J21" s="1" t="s">
@@ -2928,23 +2937,23 @@
       <c r="B22" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="14"/>
-      <c r="D22" s="23" t="s">
+      <c r="C22" s="22"/>
+      <c r="D22" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="E22" s="23" t="s">
+      <c r="E22" s="16" t="s">
         <v>220</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="14" t="s">
         <v>267</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H22" s="23" t="s">
+      <c r="H22" s="16" t="s">
         <v>223</v>
       </c>
-      <c r="I22" s="23" t="s">
+      <c r="I22" s="16" t="s">
         <v>223</v>
       </c>
       <c r="J22" s="9" t="s">
@@ -2959,23 +2968,23 @@
       <c r="B23" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="23" t="s">
+      <c r="C23" s="22"/>
+      <c r="D23" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="E23" s="23" t="s">
+      <c r="E23" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="F23" s="18" t="s">
+      <c r="F23" s="14" t="s">
         <v>268</v>
       </c>
-      <c r="G23" s="18" t="s">
+      <c r="G23" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="H23" s="23" t="s">
+      <c r="H23" s="16" t="s">
         <v>221</v>
       </c>
-      <c r="I23" s="23" t="s">
+      <c r="I23" s="16" t="s">
         <v>221</v>
       </c>
       <c r="J23" s="11" t="s">
@@ -2990,23 +2999,23 @@
       <c r="B24" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C24" s="14"/>
-      <c r="D24" s="23" t="s">
+      <c r="C24" s="22"/>
+      <c r="D24" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="E24" s="23" t="s">
+      <c r="E24" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="F24" s="18" t="s">
+      <c r="F24" s="14" t="s">
         <v>266</v>
       </c>
-      <c r="G24" s="18" t="s">
+      <c r="G24" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="H24" s="23" t="s">
+      <c r="H24" s="16" t="s">
         <v>221</v>
       </c>
-      <c r="I24" s="23" t="s">
+      <c r="I24" s="16" t="s">
         <v>221</v>
       </c>
       <c r="J24" s="11" t="s">
@@ -3021,11 +3030,11 @@
       <c r="B25" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="23" t="s">
+      <c r="C25" s="22"/>
+      <c r="D25" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="E25" s="23" t="s">
+      <c r="E25" s="16" t="s">
         <v>211</v>
       </c>
       <c r="F25" s="13" t="s">
@@ -3034,10 +3043,10 @@
       <c r="G25" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H25" s="18" t="s">
+      <c r="H25" s="14" t="s">
         <v>225</v>
       </c>
-      <c r="I25" s="23" t="s">
+      <c r="I25" s="16" t="s">
         <v>225</v>
       </c>
       <c r="J25" s="9" t="s">
@@ -3052,23 +3061,23 @@
       <c r="B26" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C26" s="14"/>
-      <c r="D26" s="23" t="s">
+      <c r="C26" s="22"/>
+      <c r="D26" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="E26" s="23" t="s">
+      <c r="E26" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="F26" s="18" t="s">
+      <c r="F26" s="14" t="s">
         <v>269</v>
       </c>
-      <c r="G26" s="18" t="s">
+      <c r="G26" s="14" t="s">
         <v>228</v>
       </c>
-      <c r="H26" s="23" t="s">
+      <c r="H26" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="I26" s="23" t="s">
+      <c r="I26" s="16" t="s">
         <v>226</v>
       </c>
       <c r="J26" s="9" t="s">
@@ -3083,11 +3092,11 @@
       <c r="B27" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C27" s="14"/>
-      <c r="D27" s="23" t="s">
+      <c r="C27" s="22"/>
+      <c r="D27" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="E27" s="23" t="s">
+      <c r="E27" s="16" t="s">
         <v>211</v>
       </c>
       <c r="F27" s="13" t="s">
@@ -3096,10 +3105,10 @@
       <c r="G27" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H27" s="18" t="s">
+      <c r="H27" s="14" t="s">
         <v>225</v>
       </c>
-      <c r="I27" s="18" t="s">
+      <c r="I27" s="14" t="s">
         <v>225</v>
       </c>
       <c r="J27" s="10" t="s">
@@ -3114,11 +3123,11 @@
       <c r="B28" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C28" s="14"/>
-      <c r="D28" s="23" t="s">
+      <c r="C28" s="22"/>
+      <c r="D28" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="E28" s="23" t="s">
+      <c r="E28" s="16" t="s">
         <v>233</v>
       </c>
       <c r="F28" s="13" t="s">
@@ -3127,10 +3136,10 @@
       <c r="G28" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H28" s="23" t="s">
+      <c r="H28" s="16" t="s">
         <v>247</v>
       </c>
-      <c r="I28" s="23" t="s">
+      <c r="I28" s="16" t="s">
         <v>248</v>
       </c>
       <c r="J28" s="10" t="s">
@@ -3147,11 +3156,11 @@
       <c r="B29" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C29" s="14"/>
-      <c r="D29" s="23" t="s">
+      <c r="C29" s="22"/>
+      <c r="D29" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="E29" s="23" t="s">
+      <c r="E29" s="16" t="s">
         <v>211</v>
       </c>
       <c r="F29" s="13" t="s">
@@ -3160,10 +3169,10 @@
       <c r="G29" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H29" s="23" t="s">
+      <c r="H29" s="16" t="s">
         <v>238</v>
       </c>
-      <c r="I29" s="23" t="s">
+      <c r="I29" s="16" t="s">
         <v>238</v>
       </c>
       <c r="J29" s="11" t="s">
@@ -3178,23 +3187,23 @@
       <c r="B30" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C30" s="14"/>
-      <c r="D30" s="23" t="s">
+      <c r="C30" s="22"/>
+      <c r="D30" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="E30" s="23" t="s">
+      <c r="E30" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="F30" s="18" t="s">
+      <c r="F30" s="14" t="s">
         <v>230</v>
       </c>
-      <c r="G30" s="23" t="s">
+      <c r="G30" s="16" t="s">
         <v>231</v>
       </c>
-      <c r="H30" s="23" t="s">
+      <c r="H30" s="16" t="s">
         <v>232</v>
       </c>
-      <c r="I30" s="23" t="s">
+      <c r="I30" s="16" t="s">
         <v>232</v>
       </c>
       <c r="J30" s="11" t="s">
@@ -3209,11 +3218,11 @@
       <c r="B31" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C31" s="14"/>
-      <c r="D31" s="23" t="s">
+      <c r="C31" s="22"/>
+      <c r="D31" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="E31" s="23" t="s">
+      <c r="E31" s="16" t="s">
         <v>233</v>
       </c>
       <c r="F31" s="13" t="s">
@@ -3222,10 +3231,10 @@
       <c r="G31" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H31" s="23" t="s">
+      <c r="H31" s="16" t="s">
         <v>235</v>
       </c>
-      <c r="I31" s="23" t="s">
+      <c r="I31" s="16" t="s">
         <v>236</v>
       </c>
       <c r="J31" s="11" t="s">
@@ -3242,11 +3251,11 @@
       <c r="B32" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C32" s="14"/>
-      <c r="D32" s="23" t="s">
+      <c r="C32" s="22"/>
+      <c r="D32" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="E32" s="23" t="s">
+      <c r="E32" s="16" t="s">
         <v>211</v>
       </c>
       <c r="F32" s="13" t="s">
@@ -3255,10 +3264,10 @@
       <c r="G32" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H32" s="23" t="s">
+      <c r="H32" s="16" t="s">
         <v>239</v>
       </c>
-      <c r="I32" s="23" t="s">
+      <c r="I32" s="16" t="s">
         <v>239</v>
       </c>
       <c r="J32" s="11" t="s">
@@ -3273,11 +3282,11 @@
       <c r="B33" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C33" s="14"/>
-      <c r="D33" s="23" t="s">
+      <c r="C33" s="22"/>
+      <c r="D33" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="E33" s="23" t="s">
+      <c r="E33" s="16" t="s">
         <v>240</v>
       </c>
       <c r="F33" s="13" t="s">
@@ -3286,10 +3295,10 @@
       <c r="G33" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H33" s="23" t="s">
+      <c r="H33" s="16" t="s">
         <v>232</v>
       </c>
-      <c r="I33" s="23" t="s">
+      <c r="I33" s="16" t="s">
         <v>232</v>
       </c>
       <c r="J33" s="11" t="s">
@@ -3304,23 +3313,23 @@
       <c r="B34" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C34" s="14"/>
-      <c r="D34" s="23" t="s">
+      <c r="C34" s="22"/>
+      <c r="D34" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="E34" s="24" t="s">
+      <c r="E34" s="17" t="s">
         <v>216</v>
       </c>
-      <c r="F34" s="18" t="s">
+      <c r="F34" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="G34" s="23" t="s">
+      <c r="G34" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="H34" s="23" t="s">
+      <c r="H34" s="16" t="s">
         <v>242</v>
       </c>
-      <c r="I34" s="23" t="s">
+      <c r="I34" s="16" t="s">
         <v>242</v>
       </c>
       <c r="J34" s="11" t="s">
@@ -3335,23 +3344,23 @@
       <c r="B35" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C35" s="14"/>
-      <c r="D35" s="23" t="s">
+      <c r="C35" s="22"/>
+      <c r="D35" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="E35" s="24" t="s">
+      <c r="E35" s="17" t="s">
         <v>216</v>
       </c>
-      <c r="F35" s="23" t="s">
+      <c r="F35" s="16" t="s">
         <v>243</v>
       </c>
       <c r="G35" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H35" s="23" t="s">
+      <c r="H35" s="16" t="s">
         <v>244</v>
       </c>
-      <c r="I35" s="23" t="s">
+      <c r="I35" s="16" t="s">
         <v>244</v>
       </c>
       <c r="J35" s="11" t="s">
@@ -3366,25 +3375,25 @@
       <c r="B36" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C36" s="14" t="s">
+      <c r="C36" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="D36" s="23" t="s">
+      <c r="D36" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="E36" s="23" t="s">
+      <c r="E36" s="16" t="s">
         <v>245</v>
       </c>
-      <c r="F36" s="18" t="s">
+      <c r="F36" s="14" t="s">
         <v>249</v>
       </c>
       <c r="G36" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H36" s="23" t="s">
+      <c r="H36" s="16" t="s">
         <v>250</v>
       </c>
-      <c r="I36" s="23" t="s">
+      <c r="I36" s="16" t="s">
         <v>250</v>
       </c>
       <c r="J36" s="11" t="s">
@@ -3399,29 +3408,31 @@
       <c r="B37" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C37" s="14"/>
-      <c r="D37" s="23" t="s">
+      <c r="C37" s="22"/>
+      <c r="D37" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="E37" s="23" t="s">
+      <c r="E37" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="F37" s="18" t="s">
+      <c r="F37" s="14" t="s">
         <v>271</v>
       </c>
       <c r="G37" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H37" s="18" t="s">
+      <c r="H37" s="14" t="s">
         <v>281</v>
       </c>
-      <c r="I37" s="18" t="s">
+      <c r="I37" s="14" t="s">
         <v>281</v>
       </c>
       <c r="J37" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="K37" s="1"/>
+      <c r="K37" s="1" t="s">
+        <v>283</v>
+      </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
@@ -3430,23 +3441,23 @@
       <c r="B38" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C38" s="14"/>
-      <c r="D38" s="23" t="s">
+      <c r="C38" s="22"/>
+      <c r="D38" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="E38" s="23" t="s">
+      <c r="E38" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="F38" s="23" t="s">
+      <c r="F38" s="16" t="s">
         <v>246</v>
       </c>
       <c r="G38" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H38" s="23" t="s">
+      <c r="H38" s="16" t="s">
         <v>251</v>
       </c>
-      <c r="I38" s="23" t="s">
+      <c r="I38" s="16" t="s">
         <v>251</v>
       </c>
       <c r="J38" s="11" t="s">
@@ -3461,23 +3472,23 @@
       <c r="B39" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C39" s="14"/>
-      <c r="D39" s="23" t="s">
+      <c r="C39" s="22"/>
+      <c r="D39" s="16" t="s">
         <v>97</v>
       </c>
       <c r="E39" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="F39" s="18" t="s">
+      <c r="F39" s="14" t="s">
         <v>272</v>
       </c>
       <c r="G39" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="H39" s="23" t="s">
+      <c r="H39" s="16" t="s">
         <v>252</v>
       </c>
-      <c r="I39" s="23" t="s">
+      <c r="I39" s="16" t="s">
         <v>252</v>
       </c>
       <c r="J39" s="11" t="s">
@@ -3487,12 +3498,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="C36:C39"/>
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="C6:C12"/>
     <mergeCell ref="C13:C14"/>
     <mergeCell ref="C15:C35"/>
-    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="J3:J39">
@@ -3532,7 +3543,7 @@
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="23" t="s">
         <v>125</v>
       </c>
       <c r="B1" s="4" t="s">
@@ -3543,7 +3554,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="16"/>
+      <c r="A2" s="24"/>
       <c r="B2" s="5" t="s">
         <v>128</v>
       </c>
@@ -3552,7 +3563,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="16"/>
+      <c r="A3" s="24"/>
       <c r="B3" s="6" t="s">
         <v>130</v>
       </c>
@@ -3561,7 +3572,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="16"/>
+      <c r="A4" s="24"/>
       <c r="B4" s="1" t="s">
         <v>132</v>
       </c>
@@ -3570,7 +3581,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" ht="33" x14ac:dyDescent="0.3">
-      <c r="A5" s="17"/>
+      <c r="A5" s="25"/>
       <c r="B5" s="7" t="s">
         <v>134</v>
       </c>

</xml_diff>